<commit_message>
Porównanie metod na wspólnym zakresie wierszy i poprawki po recenzji
- Porównanie z kluczem zawęża klucz, reguły, AI i kartę grupy do zakresu,
  który oceniało AI (domyślnie); wcześniej czułość AI liczono względem
  całego klucza, choć AI widziało tylko wybrane wiersze.
- Decyzja „pozostaw bez zmiany” nie jest alarmem; aplikacja ocenia ją osobno.
- Przycisk „Przywróć domyślne polecenie” do sprawdzenia poprawki na nowym dokumencie.
- Słownik danych w Excelu: szerokie kolumny i zawijanie tekstu (wartości bez zmian).
- Instrukcja: osobna karta po przeglądzie ręcznym, dokument kontrolny w ćw. 3,
  reguły protokołu (SBRT, uproszczony Phoenix), zasady kodowania klucza,
  zatwierdzone środowisko zamiast „tylko lokalnie”.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/exercises/dane/slownik_danych.xlsx
+++ b/exercises/dane/slownik_danych.xlsx
@@ -57,9 +57,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -428,16 +431,16 @@
   <dimension ref="A1:J35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
+    <col width="44" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -493,1354 +496,1420 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>patient_id</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Kod pacjenta</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>tekst</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>pusta komórka; w ekstrakcji null</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>pusta komórka; w ekstrakcji null</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>PR-001..PR-120; unikalny, bez identyfikatora osobowego.</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Dodatkowy duplikat pod PR-121 jest błędem struktury kohorty.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>sex</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Płeć</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>kategoria</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>pusta komórka; w ekstrakcji null</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>pusta komórka; w ekstrakcji null</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Wartość zgodna z typem, jednostką i zakresem słownika.</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>Próg kontroli jakości, nie próg rozpoznania klinicznego.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>birth_date</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Data urodzenia</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>data</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>RRRR-MM-DD</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>pusta komórka; w ekstrakcji null</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>pusta komórka; w ekstrakcji null</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Pełna data ISO; wiek w dniu RT 18–105 lat.</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>Typowa kohorta 55–85 lat; 89 lat jest dozwolone.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>diagnosis_date</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Data rozpoznania</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>data</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>RRRR-MM-DD</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>pusta komórka; w ekstrakcji null</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
+      <c r="F5" s="2" t="n"/>
+      <c r="G5" s="2" t="n"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>pusta komórka; w ekstrakcji null</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Data ISO nie późniejsza niż rozpoczęcie RT.</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>Rozpoznanie przed leczeniem radykalnym.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>rt_start_date</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Pierwsza frakcja RT</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>data</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>RRRR-MM-DD</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>pusta komórka; w ekstrakcji null</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>pusta komórka; w ekstrakcji null</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Data pierwszej frakcji w ISO.</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>Nie mylić z datą kwalifikacji ani rozpoczęcia ADT.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>weight_kg</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Masa ciała</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>liczba</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="F7" t="n">
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7" s="2" t="n">
         <v>220</v>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>pusta komórka; w ekstrakcji null</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>pusta komórka; w ekstrakcji null</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Wartość zgodna z typem, jednostką i zakresem słownika.</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Próg kontroli jakości, nie próg rozpoznania klinicznego.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>psa_dx_ng_ml</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>PSA przy rozpoznaniu</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>liczba</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>ng/ml</t>
         </is>
       </c>
-      <c r="F8" t="n">
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G8" s="2" t="n">
         <v>500</v>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>pusta komórka; w ekstrakcji null</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>pusta komórka; w ekstrakcji null</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Wartość zgodna z typem, jednostką i zakresem słownika.</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>Próg kontroli jakości, nie próg rozpoznania klinicznego.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>gleason_primary</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>Dominujący wzorzec Gleasona</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>liczba_calkowita</t>
         </is>
       </c>
-      <c r="F9" t="n">
+      <c r="D9" s="2" t="n"/>
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>pusta komórka; w ekstrakcji null</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>pusta komórka; w ekstrakcji null</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>Wartość zgodna z typem, jednostką i zakresem słownika.</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>Próg kontroli jakości, nie próg rozpoznania klinicznego.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>gleason_secondary</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Drugorzędny wzorzec Gleasona</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>liczba_calkowita</t>
         </is>
       </c>
-      <c r="F10" t="n">
+      <c r="D10" s="2" t="n"/>
+      <c r="E10" s="2" t="n"/>
+      <c r="F10" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G10" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>pusta komórka; w ekstrakcji null</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>pusta komórka; w ekstrakcji null</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Wartość zgodna z typem, jednostką i zakresem słownika.</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>Próg kontroli jakości, nie próg rozpoznania klinicznego.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>gleason_score</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Suma Gleasona</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>liczba_calkowita</t>
         </is>
       </c>
-      <c r="F11" t="n">
+      <c r="D11" s="2" t="n"/>
+      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G11" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>pusta komórka; w ekstrakcji null</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>pusta komórka; w ekstrakcji null</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>gleason_score = gleason_primary + gleason_secondary.</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>Autokonwersja 3-4 w datę nie jest wynikiem histopatologicznym.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>isup_grade</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>Grupa stopnia ISUP</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>liczba_calkowita</t>
         </is>
       </c>
-      <c r="F12" t="n">
+      <c r="D12" s="2" t="n"/>
+      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G12" t="n">
+      <c r="G12" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>pusta komórka; w ekstrakcji null</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>pusta komórka; w ekstrakcji null</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>3+3: 1; 3+4: 2; 4+3: 3; suma 8: 4; suma 9–10: 5.</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>Rozbieżność między opisem wzorców a ISUP wymaga weryfikacji preparatów lub aneksu.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>ct_stage</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>Kliniczne T</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>kategoria</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>T1c|T2a|T2b|T2c|T3a|T3b|T4</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>pusta komórka; w ekstrakcji null</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
+      <c r="F13" s="2" t="n"/>
+      <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>pusta komórka; w ekstrakcji null</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Wartość zgodna z typem, jednostką i zakresem słownika.</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>Próg kontroli jakości, nie próg rozpoznania klinicznego.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>cn_stage</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>Kliniczne N</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>kategoria</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>N0|N1</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>pusta komórka; w ekstrakcji null</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="n"/>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>pusta komórka; w ekstrakcji null</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>Wartość zgodna z typem, jednostką i zakresem słownika.</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>Próg kontroli jakości, nie próg rozpoznania klinicznego.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>risk_group</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>Grupa ryzyka wg protokołu</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>kategoria</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="D15" s="2" t="n"/>
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>niskie|posrednie|wysokie</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>pusta komórka; w ekstrakcji null</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
+      <c r="F15" s="2" t="n"/>
+      <c r="G15" s="2" t="n"/>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>pusta komórka; w ekstrakcji null</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
         <is>
           <t>Najpierw wysokie: PSA &gt;20 lub ISUP 4–5 lub cT2c–cT4 lub cN1. Następnie niskie: PSA &lt;10, ISUP 1, cT1c–cT2a i cN0. Pozostałe: posrednie. Definicja uproszczona do ćwiczenia; M1 poza rejestrem.</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="J15" s="2" t="inlineStr">
         <is>
           <t>Uproszczenie dydaktyczne; nie pełny algorytm EAU.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>rt_technique</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>Technika RT</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>kategoria</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>IMRT|VMAT|SBRT</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>pusta komórka; w ekstrakcji null</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>pusta komórka; w ekstrakcji null</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>IMRT, VMAT lub SBRT; SBRT ⇔ 5 frakcji.</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>Nie normalizować nieznanej techniki bez źródła.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>rt_dose_gy</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>Dawka na prostatę</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>liczba</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>Gy</t>
         </is>
       </c>
-      <c r="F17" t="n">
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G17" t="n">
+      <c r="G17" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>pusta komórka; w ekstrakcji null</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>pusta komórka; w ekstrakcji null</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>78/39, 76/38, 60/20, 62/20, 70/28, 36,25/5 i 40/5 (Gy/fr.). SBRT wtedy i tylko wtedy, gdy 5 frakcji.</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>Dawka całkowita na prostatę, nie dawka na węzły. 36,25/5 jest poprawne.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>rt_fractions</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>Liczba frakcji na prostatę</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>liczba_calkowita</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>fr.</t>
         </is>
       </c>
-      <c r="F18" t="n">
+      <c r="E18" s="2" t="n"/>
+      <c r="F18" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G18" t="n">
+      <c r="G18" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>pusta komórka; w ekstrakcji null</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>pusta komórka; w ekstrakcji null</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>78/39, 76/38, 60/20, 62/20, 70/28, 36,25/5 i 40/5 (Gy/fr.). SBRT wtedy i tylko wtedy, gdy 5 frakcji.</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>Pole nie obejmuje osobnej liczby frakcji obszaru węzłowego.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>adt</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>Stosowanie ADT</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>logiczna</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>0|1</t>
         </is>
       </c>
-      <c r="F19" t="n">
+      <c r="F19" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G19" t="n">
+      <c r="G19" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>pusta komórka; w ekstrakcji null</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>pusta komórka; w ekstrakcji null</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>adt=0 wymaga adt_months=0. ADT 6 mies. typowo w ryzyku pośrednim niekorzystnym; 18–36 mies. w wysokim. adt_months: całkowity zaplanowany czas ADT.</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="J19" s="2" t="inlineStr">
         <is>
           <t>0 oznacza udokumentowane niestosowanie; brak wzmianki to null.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>adt_months</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>Zaplanowany czas ADT</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>liczba_calkowita</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>mies.</t>
         </is>
       </c>
-      <c r="F20" t="n">
+      <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G20" t="n">
+      <c r="G20" s="2" t="n">
         <v>36</v>
       </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>pusta komórka; w ekstrakcji null</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>pusta komórka; w ekstrakcji null</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>adt=0 wymaga adt_months=0. ADT 6 mies. typowo w ryzyku pośrednim niekorzystnym; 18–36 mies. w wysokim. adt_months: całkowity zaplanowany czas ADT.</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="J20" s="2" t="inlineStr">
         <is>
           <t>Czas zaplanowany, nie czas od pierwszego podania do pobrania krwi.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>testosterone_ng_dl</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>Testosteron</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>liczba</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>ng/dl</t>
         </is>
       </c>
-      <c r="F21" t="n">
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G21" t="n">
+      <c r="G21" s="2" t="n">
         <v>1200</v>
       </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>pusta komórka; w ekstrakcji null</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>pusta komórka; w ekstrakcji null</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
         <is>
           <t>0–1200 ng/dl; nmol/l × 28,84.</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="J21" s="2" t="inlineStr">
         <is>
           <t>180 ng/dl w pierwszym miesiącu ADT to dopuszczalna pułapka. Sama liczba nie identyfikuje jednostki.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>psa_nadir_ng_ml</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>Nadir PSA po RT</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>liczba</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>ng/ml</t>
         </is>
       </c>
-      <c r="F22" t="n">
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G22" t="n">
+      <c r="G22" s="2" t="n">
         <v>500</v>
       </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>pusta komórka; w ekstrakcji null</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>pusta komórka; w ekstrakcji null</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
         <is>
           <t>Nadir ≤ ostatnie PSA; &lt;0,01 wymaga jawnego sposobu kodowania wyników cenzorowanych.</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="J22" s="2" t="inlineStr">
         <is>
           <t>Nie podstawiać zera ani połowy granicy oznaczalności.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>psa_last_ng_ml</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>Ostatnie PSA</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>liczba</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>ng/ml</t>
         </is>
       </c>
-      <c r="F23" t="n">
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G23" t="n">
+      <c r="G23" s="2" t="n">
         <v>500</v>
       </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>pusta komórka; w ekstrakcji null</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>pusta komórka; w ekstrakcji null</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
         <is>
           <t>Wartość zgodna z typem, jednostką i zakresem słownika.</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="J23" s="2" t="inlineStr">
         <is>
           <t>Próg kontroli jakości, nie próg rozpoznania klinicznego.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>psa_last_date</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>Data ostatniego PSA</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>data</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="D24" s="2" t="n"/>
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>RRRR-MM-DD</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>pusta komórka; w ekstrakcji null</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="n"/>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>pusta komórka; w ekstrakcji null</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
         <is>
           <t>ISO; po rozpoczęciu RT i przed datą zgonu.</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="J24" s="2" t="inlineStr">
         <is>
           <t>Phoenix nie rozstrzyga etiologii wzrostu PSA.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>bcr_phoenix</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>Nawrót wg Phoenix</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>logiczna</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>0|1</t>
         </is>
       </c>
-      <c r="F25" t="n">
+      <c r="F25" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G25" t="n">
+      <c r="G25" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>pusta komórka; w ekstrakcji null</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>pusta komórka; w ekstrakcji null</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
         <is>
           <t>bcr_phoenix = 1, gdy PSA ostatnie &gt;= nadir + 2 ng/ml; inaczej 0. Bez obu pomiarów: null.</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr">
+      <c r="J25" s="2" t="inlineStr">
         <is>
           <t>Definicja protokołu ćwiczeniowego.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>gu_toxicity_max</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>Maksymalna toksyczność GU</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>liczba_calkowita</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>CTCAE</t>
         </is>
       </c>
-      <c r="F26" t="n">
+      <c r="E26" s="2" t="n"/>
+      <c r="F26" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G26" t="n">
+      <c r="G26" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>pusta komórka; w ekstrakcji null</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>pusta komórka; w ekstrakcji null</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
         <is>
           <t>Całkowite 0–5 CTCAE; maksimum całej obserwacji.</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="J26" s="2" t="inlineStr">
         <is>
           <t>Pojedyncze G3 jest prawdziwe i nie podlega usunięciu.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>gi_toxicity_max</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>Maksymalna toksyczność GI</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr">
         <is>
           <t>liczba_calkowita</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>CTCAE</t>
         </is>
       </c>
-      <c r="F27" t="n">
+      <c r="E27" s="2" t="n"/>
+      <c r="F27" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G27" t="n">
+      <c r="G27" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>pusta komórka; w ekstrakcji null</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>pusta komórka; w ekstrakcji null</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
         <is>
           <t>Całkowite 0–5 CTCAE; maksimum całej obserwacji.</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="J27" s="2" t="inlineStr">
         <is>
           <t>Brak wzmianki o toksyczności nie oznacza G0.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>creatinine_mg_dl</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>Kreatynina</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>liczba</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>mg/dl</t>
         </is>
       </c>
-      <c r="F28" t="n">
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="n">
         <v>0.2</v>
       </c>
-      <c r="G28" t="n">
+      <c r="G28" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>pusta komórka; w ekstrakcji null</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>pusta komórka; w ekstrakcji null</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
         <is>
           <t>0,2–15 mg/dl; µmol/l ÷ 88,4.</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="J28" s="2" t="inlineStr">
         <is>
           <t>Inną jednostkę potwierdzić, jeśli nie zapisano jej w komórce lub dokumencie.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>hemoglobin_g_dl</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>Hemoglobina</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>liczba</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>g/dl</t>
         </is>
       </c>
-      <c r="F29" t="n">
+      <c r="E29" s="2" t="n"/>
+      <c r="F29" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G29" t="n">
+      <c r="G29" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>pusta komórka; w ekstrakcji null</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>pusta komórka; w ekstrakcji null</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
         <is>
           <t>5–20 g/dl; mmol/l ÷ 0,6206.</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="J29" s="2" t="inlineStr">
         <is>
           <t>8,4 może być prawdziwą anemią albo inną jednostką; sama liczba nie rozstrzyga.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>diabetes</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>Cukrzyca</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>logiczna</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="D30" s="2" t="n"/>
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>0|1</t>
         </is>
       </c>
-      <c r="F30" t="n">
+      <c r="F30" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G30" t="n">
+      <c r="G30" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>pusta komórka; w ekstrakcji null</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>pusta komórka; w ekstrakcji null</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
         <is>
           <t>0/1 według udokumentowanego wywiadu.</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="J30" s="2" t="inlineStr">
         <is>
           <t>Brak informacji = null, nie 0.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>hypertension</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>Nadciśnienie tętnicze</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>logiczna</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="D31" s="2" t="n"/>
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>0|1</t>
         </is>
       </c>
-      <c r="F31" t="n">
+      <c r="F31" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G31" t="n">
+      <c r="G31" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>pusta komórka; w ekstrakcji null</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>pusta komórka; w ekstrakcji null</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
         <is>
           <t>0/1 według udokumentowanego wywiadu.</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="J31" s="2" t="inlineStr">
         <is>
           <t>Pojedynczy pomiar ciśnienia nie rozstrzyga rozpoznania.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>smoking</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>Palenie</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>kategoria</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="D32" s="2" t="n"/>
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>never|former|current</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>pusta komórka; w ekstrakcji null</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
+      <c r="F32" s="2" t="n"/>
+      <c r="G32" s="2" t="n"/>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>pusta komórka; w ekstrakcji null</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
         <is>
           <t>never/former/current.</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="J32" s="2" t="inlineStr">
         <is>
           <t>Nie pali od 10 lat = former; samo nie pali nie rozstrzyga never/former.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>death</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>Zgon</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>logiczna</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="D33" s="2" t="n"/>
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>0|1</t>
         </is>
       </c>
-      <c r="F33" t="n">
+      <c r="F33" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G33" t="n">
+      <c r="G33" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>pusta komórka; w ekstrakcji null</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>pusta komórka; w ekstrakcji null</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
         <is>
           <t>1 wymaga daty zgonu; 0 wymaga pustej daty.</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="J33" s="2" t="inlineStr">
         <is>
           <t>Nie wolno ustalać statusu z samego braku daty.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>death_date</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>Data zgonu</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>data</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="D34" s="2" t="n"/>
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>RRRR-MM-DD</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>pusta komórka; w ekstrakcji null</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
+      <c r="F34" s="2" t="n"/>
+      <c r="G34" s="2" t="n"/>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>pusta komórka; w ekstrakcji null</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
         <is>
           <t>ISO; po rozpoczęciu RT i nie przed ostatnim PSA.</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr">
+      <c r="J34" s="2" t="inlineStr">
         <is>
           <t>Pusta komórka poprawna wyłącznie przy death=0.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>Uwagi</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>tekst</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>pusta komórka; w ekstrakcji null</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
+      <c r="D35" s="2" t="n"/>
+      <c r="E35" s="2" t="n"/>
+      <c r="F35" s="2" t="n"/>
+      <c r="G35" s="2" t="n"/>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>pusta komórka; w ekstrakcji null</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
         <is>
           <t>Bez PESEL; rozproszone dane strukturalne przenieść po uzgodnieniu.</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr">
+      <c r="J35" s="2" t="inlineStr">
         <is>
           <t>Nie rozpoznawać cukrzycy wyłącznie na podstawie nazwy leku.</t>
         </is>

</xml_diff>